<commit_message>
Added solving for x,y,..., commented a bit, updated the BOM, and removed video so I can upload it for the next git commit very soon
</commit_message>
<xml_diff>
--- a/BOM_calculator.xlsx
+++ b/BOM_calculator.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="112">
   <si>
     <t xml:space="preserve">No.</t>
   </si>
@@ -52,6 +52,9 @@
     <t xml:space="preserve">Supplier</t>
   </si>
   <si>
+    <t xml:space="preserve">JLCPCB Unit Price</t>
+  </si>
+  <si>
     <t xml:space="preserve">JLCPCB Price</t>
   </si>
   <si>
@@ -89,6 +92,7 @@
         <color theme="1"/>
         <rFont val="Arial Unicode MS"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">村田</t>
     </r>
@@ -110,9 +114,6 @@
     <t xml:space="preserve">LCSC</t>
   </si>
   <si>
-    <t xml:space="preserve">0.0171</t>
-  </si>
-  <si>
     <t xml:space="preserve">42714</t>
   </si>
   <si>
@@ -147,6 +148,7 @@
         <color theme="1"/>
         <rFont val="Arial Unicode MS"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">三星</t>
     </r>
@@ -165,9 +167,6 @@
     <t xml:space="preserve">C86295</t>
   </si>
   <si>
-    <t xml:space="preserve">0.0024</t>
-  </si>
-  <si>
     <t xml:space="preserve">8697</t>
   </si>
   <si>
@@ -186,9 +185,6 @@
     <t xml:space="preserve">C29936</t>
   </si>
   <si>
-    <t xml:space="preserve">0.0011</t>
-  </si>
-  <si>
     <t xml:space="preserve">2742739</t>
   </si>
   <si>
@@ -220,6 +216,7 @@
         <color theme="1"/>
         <rFont val="Arial Unicode MS"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">安世</t>
     </r>
@@ -238,9 +235,6 @@
     <t xml:space="preserve">C24372</t>
   </si>
   <si>
-    <t xml:space="preserve">0.0031</t>
-  </si>
-  <si>
     <t xml:space="preserve">90588</t>
   </si>
   <si>
@@ -272,6 +266,7 @@
         <color theme="1"/>
         <rFont val="Arial Unicode MS"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">聚兴泰</t>
     </r>
@@ -290,9 +285,6 @@
     <t xml:space="preserve">C42431809</t>
   </si>
   <si>
-    <t xml:space="preserve">0.0058</t>
-  </si>
-  <si>
     <t xml:space="preserve">4744</t>
   </si>
   <si>
@@ -324,6 +316,7 @@
         <color theme="1"/>
         <rFont val="Arial Unicode MS"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">韩下</t>
     </r>
@@ -342,16 +335,25 @@
     <t xml:space="preserve">C50878477</t>
   </si>
   <si>
-    <t xml:space="preserve">0.0213</t>
-  </si>
-  <si>
     <t xml:space="preserve">7</t>
   </si>
   <si>
+    <t xml:space="preserve">Custom Power PCB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P1</t>
+  </si>
+  <si>
     <t xml:space="preserve">ESP32-3.3V and sense</t>
   </si>
   <si>
-    <t xml:space="preserve">P1</t>
+    <t xml:space="preserve">XXXXXXXXXXXX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ordered by user</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aliexpress</t>
   </si>
   <si>
     <t xml:space="preserve">8</t>
@@ -406,6 +408,7 @@
         <color theme="1"/>
         <rFont val="Arial Unicode MS"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">时科</t>
     </r>
@@ -424,9 +427,6 @@
     <t xml:space="preserve">C475630</t>
   </si>
   <si>
-    <t xml:space="preserve">0.0021</t>
-  </si>
-  <si>
     <t xml:space="preserve">50985</t>
   </si>
   <si>
@@ -461,6 +461,7 @@
         <color theme="1"/>
         <rFont val="Arial Unicode MS"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">国巨</t>
     </r>
@@ -479,9 +480,6 @@
     <t xml:space="preserve">C98220</t>
   </si>
   <si>
-    <t xml:space="preserve">0.0003</t>
-  </si>
-  <si>
     <t xml:space="preserve">49</t>
   </si>
   <si>
@@ -513,6 +511,7 @@
         <color theme="1"/>
         <rFont val="Arial Unicode MS"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">品赞</t>
     </r>
@@ -531,9 +530,6 @@
     <t xml:space="preserve">C29780122</t>
   </si>
   <si>
-    <t xml:space="preserve">0.002</t>
-  </si>
-  <si>
     <t xml:space="preserve">177811</t>
   </si>
   <si>
@@ -565,6 +561,7 @@
         <color theme="1"/>
         <rFont val="Arial Unicode MS"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">摩天射频</t>
     </r>
@@ -583,9 +580,6 @@
     <t xml:space="preserve">C22467599</t>
   </si>
   <si>
-    <t xml:space="preserve">0.0414</t>
-  </si>
-  <si>
     <t xml:space="preserve">1534</t>
   </si>
   <si>
@@ -620,6 +614,7 @@
         <color theme="1"/>
         <rFont val="Arial Unicode MS"/>
         <family val="2"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">乐鑫</t>
     </r>
@@ -638,20 +633,30 @@
     <t xml:space="preserve">C2913202</t>
   </si>
   <si>
-    <t xml:space="preserve">0.727</t>
-  </si>
-  <si>
     <t xml:space="preserve">27666</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FTDI FT232RL CH340N</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not on Board</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FT232RL CH340N</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aitver Electronics</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="General"/>
+    <numFmt numFmtId="165" formatCode="#,##0.0000\ [$€-C0A];\-#,##0.0000\ [$€-C0A]"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -693,8 +698,38 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Avenir Next"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Arial Unicode MS"/>
       <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10.5"/>
+      <color theme="1"/>
+      <name val="Avenir Next"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Avenir Next"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <i val="true"/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Avenir Next"/>
+      <family val="0"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -739,29 +774,69 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="16">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -953,532 +1028,618 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L15"/>
+  <dimension ref="A1:M15"/>
   <sheetFormatPr defaultColWidth="8.515625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6.47"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="10.01"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="31.11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="5" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="10.78"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6.47"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="10.01"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="19.1"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="31.58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="5" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="12.32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="14.17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="14.02"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="10.16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="28.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="2" t="s">
         <v>11</v>
       </c>
+      <c r="M1" s="2" t="s">
+        <v>12</v>
+      </c>
     </row>
-    <row r="2" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B2" s="3" t="n">
+    <row r="2" customFormat="false" ht="33.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="C2" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D2" s="4" t="s">
+      <c r="C2" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="D2" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="F2" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G2" s="4" t="s">
+      <c r="E2" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="F2" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G2" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="I2" s="4" t="s">
+      <c r="H2" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="J2" s="4" t="s">
+      <c r="I2" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="K2" s="4" t="s">
+      <c r="J2" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="L2" s="4" t="s">
+      <c r="K2" s="7" t="n">
+        <v>0.0171</v>
+      </c>
+      <c r="L2" s="7" t="n">
+        <f aca="false">K2*B2</f>
+        <v>0.0513</v>
+      </c>
+      <c r="M2" s="5" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="17.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+    <row r="3" customFormat="false" ht="33.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="3" t="n">
+      <c r="B3" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="F3" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="G3" s="4" t="s">
+      <c r="G3" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="H3" s="4" t="s">
+      <c r="H3" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="I3" s="4" t="s">
+      <c r="I3" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="J3" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="K3" s="4" t="s">
+      <c r="J3" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="K3" s="7" t="n">
+        <v>0.0024</v>
+      </c>
+      <c r="L3" s="7" t="n">
+        <f aca="false">K3*B3</f>
+        <v>0.0024</v>
+      </c>
+      <c r="M3" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="L3" s="4" t="s">
+    </row>
+    <row r="4" customFormat="false" ht="33.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="17.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
+      <c r="B4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="B4" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C4" s="4" t="s">
+      <c r="D4" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="E4" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="G4" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="E4" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="G4" s="4" t="s">
+      <c r="H4" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="I4" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="H4" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="I4" s="4" t="s">
+      <c r="J4" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="K4" s="7" t="n">
+        <v>0.0011</v>
+      </c>
+      <c r="L4" s="7" t="n">
+        <f aca="false">K4*B4</f>
+        <v>0.0011</v>
+      </c>
+      <c r="M4" s="5" t="s">
         <v>35</v>
-      </c>
-      <c r="J4" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="K4" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="L4" s="4" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="71.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="D5" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="B5" s="3" t="n">
+      <c r="E5" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="F5" s="6"/>
+      <c r="G5" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="K5" s="7" t="n">
+        <v>0.0031</v>
+      </c>
+      <c r="L5" s="7" t="n">
+        <f aca="false">K5*B5</f>
+        <v>0.155</v>
+      </c>
+      <c r="M5" s="5" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="64.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="F6" s="6"/>
+      <c r="G6" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="H6" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="K6" s="7" t="n">
+        <v>0.0058</v>
+      </c>
+      <c r="L6" s="7" t="n">
+        <f aca="false">K6*B6</f>
+        <v>0.0058</v>
+      </c>
+      <c r="M6" s="5" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="33.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="C5" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="H5" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="I5" s="4" t="s">
+      <c r="B7" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="F7" s="6"/>
+      <c r="G7" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="H7" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="I7" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="J7" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="K7" s="7" t="n">
+        <v>0.0213</v>
+      </c>
+      <c r="L7" s="7" t="n">
+        <f aca="false">K7*B7</f>
+        <v>0.0213</v>
+      </c>
+      <c r="M7" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="J5" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="K5" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="L5" s="4" t="s">
-        <v>45</v>
-      </c>
     </row>
-    <row r="6" customFormat="false" ht="47.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="B6" s="3" t="n">
+    <row r="8" customFormat="false" ht="33.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="B8" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="C6" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="F6" s="4"/>
-      <c r="G6" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="H6" s="4" t="s">
+      <c r="C8" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="F8" s="6"/>
+      <c r="G8" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="I8" s="6"/>
+      <c r="J8" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="K8" s="7" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="L8" s="7" t="n">
+        <f aca="false">K8*B8</f>
+        <v>8.5</v>
+      </c>
+      <c r="M8" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="33.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="F9" s="6"/>
+      <c r="G9" s="6"/>
+      <c r="H9" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="I9" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="J9" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="K9" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="L9" s="7" t="n">
+        <f aca="false">K9*B9</f>
+        <v>5</v>
+      </c>
+      <c r="M9" s="5" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="33.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="B10" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="F10" s="6"/>
+      <c r="G10" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="H10" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="I10" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="J10" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="K10" s="7" t="n">
+        <v>0.0021</v>
+      </c>
+      <c r="L10" s="7" t="n">
+        <f aca="false">K10*B10</f>
+        <v>0.0042</v>
+      </c>
+      <c r="M10" s="5" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="38.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="G11" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="H11" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="I11" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="J11" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="K11" s="7" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="L11" s="7" t="n">
+        <f aca="false">K11*B11</f>
+        <v>0.0027</v>
+      </c>
+      <c r="M11" s="5" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="106.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="B12" s="4" t="n">
         <v>50</v>
       </c>
-      <c r="I6" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="J6" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="K6" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="L6" s="4" t="s">
-        <v>53</v>
+      <c r="C12" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="F12" s="6"/>
+      <c r="G12" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="H12" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="I12" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="J12" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="K12" s="7" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="L12" s="7" t="n">
+        <f aca="false">K12*B12</f>
+        <v>0.1</v>
+      </c>
+      <c r="M12" s="5" t="s">
+        <v>92</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="B7" s="3" t="n">
+    <row r="13" customFormat="false" ht="29.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="B13" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="C7" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="F7" s="4"/>
-      <c r="G7" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="H7" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="I7" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="J7" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="K7" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="L7" s="4" t="s">
-        <v>46</v>
+      <c r="C13" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="E13" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="F13" s="6"/>
+      <c r="G13" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="H13" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="I13" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="J13" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="K13" s="7" t="n">
+        <v>0.0414</v>
+      </c>
+      <c r="L13" s="7" t="n">
+        <f aca="false">K13*B13</f>
+        <v>0.0414</v>
+      </c>
+      <c r="M13" s="5" t="s">
+        <v>99</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="B8" s="3" t="n">
+    <row r="14" customFormat="false" ht="33.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="B14" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="C8" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="F8" s="4"/>
-      <c r="G8" s="4"/>
-      <c r="H8" s="4"/>
-      <c r="I8" s="4"/>
-      <c r="J8" s="4"/>
-      <c r="K8" s="4"/>
-      <c r="L8" s="4"/>
+      <c r="C14" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="E14" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="F14" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="G14" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="H14" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="I14" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="J14" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="K14" s="7" t="n">
+        <v>0.727</v>
+      </c>
+      <c r="L14" s="7" t="n">
+        <f aca="false">K14*B14</f>
+        <v>0.727</v>
+      </c>
+      <c r="M14" s="5" t="s">
+        <v>107</v>
+      </c>
     </row>
-    <row r="9" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="B9" s="3" t="n">
+    <row r="15" customFormat="false" ht="22.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B15" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="C9" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="F9" s="4"/>
-      <c r="G9" s="4"/>
-      <c r="H9" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="I9" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="J9" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="K9" s="4"/>
-      <c r="L9" s="4" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="B10" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="F10" s="4"/>
-      <c r="G10" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="H10" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="I10" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="J10" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="K10" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="L10" s="4" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="B11" s="3" t="n">
-        <v>9</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="E11" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="F11" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="G11" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="H11" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="I11" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="J11" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="K11" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="L11" s="4" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="104" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="B12" s="3" t="n">
-        <v>50</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="F12" s="4"/>
-      <c r="G12" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="H12" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="I12" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="J12" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="K12" s="4" t="s">
-        <v>95</v>
-      </c>
-      <c r="L12" s="4" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="B13" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="E13" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="F13" s="4"/>
-      <c r="G13" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="H13" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="I13" s="4" t="s">
-        <v>102</v>
-      </c>
-      <c r="J13" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="K13" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="L13" s="4" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="B14" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="D14" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="E14" s="4" t="s">
+      <c r="C15" s="11" t="s">
         <v>108</v>
       </c>
-      <c r="F14" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="G14" s="4" t="s">
+      <c r="D15" s="12" t="s">
         <v>109</v>
       </c>
-      <c r="H14" s="4" t="s">
+      <c r="E15" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="F15" s="13"/>
+      <c r="G15" s="11" t="s">
         <v>110</v>
       </c>
-      <c r="I14" s="4" t="s">
+      <c r="H15" s="13" t="s">
         <v>111</v>
       </c>
-      <c r="J14" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="K14" s="4" t="s">
-        <v>112</v>
-      </c>
-      <c r="L14" s="4" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="5"/>
-      <c r="C15" s="5"/>
-      <c r="D15" s="5"/>
-      <c r="E15" s="5"/>
-      <c r="F15" s="5"/>
-      <c r="G15" s="5"/>
-      <c r="H15" s="5"/>
-      <c r="I15" s="5"/>
-      <c r="J15" s="5"/>
-      <c r="K15" s="5" t="n">
-        <f aca="false">SUM(B2:B14)</f>
-        <v>122</v>
-      </c>
-      <c r="L15" s="5"/>
+      <c r="I15" s="13"/>
+      <c r="J15" s="13"/>
+      <c r="K15" s="14" t="n">
+        <f aca="false">SUM(K2:K14)</f>
+        <v>14.3236</v>
+      </c>
+      <c r="L15" s="14" t="n">
+        <f aca="false">SUM(L2:L14)</f>
+        <v>14.6122</v>
+      </c>
+      <c r="M15" s="15"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="true" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>